<commit_message>
Add 5 new annotations (ORCL/INTC/MU/CRM/TSLA) + re-annotate MSFT with standard schema; expand training set to 10 samples
</commit_message>
<xml_diff>
--- a/data/extracted/core_indicators_45_v01.xlsx
+++ b/data/extracted/core_indicators_45_v01.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -484,7 +484,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>核心财务指标表 v0.1（5家公司 × 45指标）</t>
+          <t>核心财务指标表 v0.1（10家公司 × 45指标）</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-21（v0.2：从10-K原文补提35项缺口，剩余21项为公司真未披露）</t>
+          <t>2026-07-21（v0.2：从10-K原文补提35项缺口）；2026-07-22（v0.3：扩展至10家——新增ORCL/INTC/MU/CRM/TSLA，MSFT按新版标准结构标注JSON整体改写，旧版capex 55300/goodwill 118300等错误值已替换）</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>data/annotated/ 下5份已校验标注JSON（META/NVDA/AMD/GOOGL/MSFT）+ Meta团队指标清单doc</t>
+          <t>data/annotated/ 下10份已校验标注JSON（META/NVDA/AMD/GOOGL/MSFT/ORCL/INTC/MU/CRM/TSLA）+ Meta团队指标清单doc</t>
         </is>
       </c>
     </row>
@@ -544,29 +544,41 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>META ppe数据已经Note7核实（行6528，全表勾稽通过，含融资租赁ROU）；NVDA capex含无形资产购买未拆分；GOOGL servers_gross=Information technology assets、buildings_gross=Land and buildings口径；MSFT capex为additions口径、finance_lease取自Note14补充披露；AMD buildings_gross为Land+building+leasehold合并口径、intangible_assets_net仅收购相关；各家累计折旧均不按资产类别拆分（servers_net/buildings_net为真NA）</t>
+          <t>META ppe数据已经Note7核实（行6528，全表勾稽通过，含融资租赁ROU）；NVDA capex含无形资产购买未拆分；GOOGL servers_gross=Information technology assets、buildings_gross=Land and buildings口径；AMD buildings_gross为Land+building+leasehold合并口径、intangible_assets_net仅收购相关；各家累计折旧均不按资产类别拆分（servers_net/buildings_net为真NA）</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>配套文件</t>
+          <t>口径注记(v0.3新增)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>data/processed/training_v01.csv（训练用，公司×指标宽表）</t>
+          <t>MSFT capex为现金流量表additions现金口径44477（另新增融资租赁ROU 11633未计入）、折旧15200为四舍五入口径、finance_lease_payments本期NA；ORCL servers_gross=Computer/network/machinery/equipment原值、无融资租赁；INTC为IDM无servers口径（machinery 100033→equipment_gross）、accelerated_dep_charges=本期excess capacity charges 411（非折旧科目但经济性质等同闲置产能加速费用化）；MU ppe_gross 87585无服务器细分；CRM depreciation 1100为Note5固定资产口径（现金流量表合并D&amp;A 3959）；TSLA depreciation_coverage用operating_income 8891口径（净利润14974含一次性递延税转回5.93B被扭曲）</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>配套文件</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>data/processed/training_v01.csv（训练用，公司×指标宽表）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>标签说明</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>D1-D5为五维度人工评分(1-5)，composite_score为加权综合分，risk_level为风险等级</t>
         </is>
@@ -583,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -597,6 +609,10 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -650,6 +666,31 @@
           <t>MSFT</t>
         </is>
       </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -690,7 +731,21 @@
       <c r="J2" s="4" t="n">
         <v>512163</v>
       </c>
-      <c r="K2" s="4" t="n"/>
+      <c r="K2" s="4" t="n">
+        <v>140976</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>191572</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>64254</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>99823</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>106618</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -731,7 +786,21 @@
       <c r="J3" s="4" t="n">
         <v>135591</v>
       </c>
-      <c r="K3" s="4" t="n"/>
+      <c r="K3" s="4" t="n">
+        <v>21536</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>96647</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>37928</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>3689</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>29725</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -772,7 +841,21 @@
       <c r="J4" s="4" t="n">
         <v>212012</v>
       </c>
-      <c r="K4" s="4" t="n"/>
+      <c r="K4" s="4" t="n">
+        <v>34818</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>194657</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>87585</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>6841</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>41782</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -813,7 +896,21 @@
       <c r="J5" s="4" t="n">
         <v>76421</v>
       </c>
-      <c r="K5" s="4" t="n"/>
+      <c r="K5" s="4" t="n">
+        <v>13282</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>98010</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>49657</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>3152</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>12057</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -855,12 +952,28 @@
       <c r="I6" s="4" t="n">
         <v>80594</v>
       </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="n"/>
+      <c r="J6" s="4" t="n">
+        <v>93780</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>20989</v>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>4209</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>3799</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -911,7 +1024,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K7" s="4" t="n"/>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -954,7 +1091,27 @@
       <c r="J8" s="4" t="n">
         <v>93943</v>
       </c>
-      <c r="K8" s="4" t="n"/>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>51182</v>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>490</v>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1005,7 +1162,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K9" s="4" t="n"/>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1048,7 +1229,23 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K10" s="4" t="n"/>
+      <c r="K10" s="4" t="n">
+        <v>5634</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>43442</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>2464</v>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>5791</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1091,7 +1288,21 @@
       <c r="J11" s="4" t="n">
         <v>27597</v>
       </c>
-      <c r="K11" s="4" t="n"/>
+      <c r="K11" s="4" t="n">
+        <v>6890</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>4589</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>404</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>5278</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>178</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1132,7 +1343,21 @@
       <c r="J12" s="4" t="n">
         <v>119220</v>
       </c>
-      <c r="K12" s="4" t="n"/>
+      <c r="K12" s="4" t="n">
+        <v>62230</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>27591</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>1150</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>48620</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>253</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1173,7 +1398,21 @@
       <c r="J13" s="4" t="n">
         <v>245122</v>
       </c>
-      <c r="K13" s="4" t="n"/>
+      <c r="K13" s="4" t="n">
+        <v>52961</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>54228</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>15540</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>34857</v>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>96773</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1214,7 +1453,21 @@
       <c r="J14" s="4" t="n">
         <v>88136</v>
       </c>
-      <c r="K14" s="4" t="n"/>
+      <c r="K14" s="4" t="n">
+        <v>10467</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>1675</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>-5833</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>4136</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>14974</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1255,7 +1508,21 @@
       <c r="J15" s="4" t="n">
         <v>109433</v>
       </c>
-      <c r="K15" s="4" t="n"/>
+      <c r="K15" s="4" t="n">
+        <v>15353</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>93</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>-5745</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>5011</v>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>8891</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1296,7 +1563,21 @@
       <c r="J16" s="4" t="n">
         <v>19651</v>
       </c>
-      <c r="K16" s="4" t="n"/>
+      <c r="K16" s="4" t="n">
+        <v>1274</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>-913</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>177</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>814</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>-5001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1337,7 +1618,21 @@
       <c r="J17" s="4" t="n">
         <v>29510</v>
       </c>
-      <c r="K17" s="4" t="n"/>
+      <c r="K17" s="4" t="n">
+        <v>8915</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>16046</v>
+      </c>
+      <c r="M17" s="4" t="n">
+        <v>3114</v>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>4906</v>
+      </c>
+      <c r="O17" s="4" t="n">
+        <v>3969</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1375,10 +1670,36 @@
       <c r="I18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="4" t="n"/>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1419,7 +1740,25 @@
       <c r="J19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="4" t="n"/>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="M19" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1460,7 +1799,21 @@
       <c r="J20" s="4" t="n">
         <v>15200</v>
       </c>
-      <c r="K20" s="4" t="n"/>
+      <c r="K20" s="4" t="n">
+        <v>3129</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>7847</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>7670</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>1100</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>3330</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1503,7 +1856,23 @@
       <c r="J21" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="K21" s="4" t="n"/>
+      <c r="K21" s="4" t="n">
+        <v>3010</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>1755</v>
+      </c>
+      <c r="M21" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>1869</v>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1544,7 +1913,21 @@
       <c r="J22" s="4" t="n">
         <v>44477</v>
       </c>
-      <c r="K22" s="4" t="n"/>
+      <c r="K22" s="4" t="n">
+        <v>6866</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>25750</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>7676</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>736</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>8898</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1588,10 +1971,28 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="J23" s="4" t="n">
-        <v>1286</v>
-      </c>
-      <c r="K23" s="4" t="n"/>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="M23" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>629</v>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>464</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1632,7 +2033,21 @@
       <c r="J24" s="4" t="n">
         <v>118548</v>
       </c>
-      <c r="K24" s="4" t="n"/>
+      <c r="K24" s="4" t="n">
+        <v>18673</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>11471</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>1559</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>10234</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>13256</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1683,7 +2098,31 @@
           <t>6(FY2023起由4年延长)</t>
         </is>
       </c>
-      <c r="K25" s="4" t="n"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>5(FY2023 Q1由4年延长,本期无变更)</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>3-5(计算机/设备/软件)</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>3-10(计算机设备与软件)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1734,7 +2173,31 @@
           <t>5-15</t>
         </is>
       </c>
-      <c r="K26" s="4" t="n"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>1-40</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>10-25</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>10-30</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>10-40</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>15-30</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
@@ -1778,12 +2241,32 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="n"/>
+      <c r="J27" s="4" t="n">
+        <v>8163</v>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>293</v>
+      </c>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
@@ -1827,12 +2310,28 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="n"/>
+      <c r="J28" s="4" t="n">
+        <v>6532</v>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>100033</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>65555</v>
+      </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="n">
+        <v>16372</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
@@ -1883,7 +2382,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K29" s="4" t="n"/>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O29" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
@@ -1934,7 +2457,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K30" s="4" t="n"/>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
@@ -1985,7 +2532,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K31" s="4" t="n"/>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O31" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -2036,7 +2607,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K32" s="4" t="n"/>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -2087,7 +2682,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K33" s="4" t="n"/>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -2138,7 +2757,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K34" s="4" t="n"/>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
@@ -2189,7 +2832,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K35" s="4" t="n"/>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O35" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
@@ -2240,7 +2907,29 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K36" s="4" t="n"/>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>-1416</v>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
@@ -2291,7 +2980,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K37" s="4" t="n"/>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O37" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
@@ -2340,7 +3053,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K38" s="4" t="n"/>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
@@ -2389,7 +3126,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K39" s="4" t="n"/>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O39" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
@@ -2438,7 +3199,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K40" s="4" t="n"/>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O40" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
@@ -2487,7 +3272,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K41" s="4" t="n"/>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O41" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
@@ -2538,7 +3347,31 @@
           <t>2-6(计算机设备)</t>
         </is>
       </c>
-      <c r="K42" s="4" t="n"/>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>1-5(计算机/网络/机器设备)</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>3-8(2023-01部分生产设备由5延至8)</t>
+        </is>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>7(生产设备;其他≤7)</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>5(家具);租赁改良≤10</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>3-15(机器/设备/车辆/家具;tooling 4-7)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
@@ -2589,7 +3422,31 @@
           <t>3(内部使用软件)</t>
         </is>
       </c>
-      <c r="K43" s="4" t="n"/>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>3-5(随PPE软件类)</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>3-5(内部使用软件)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
@@ -2637,10 +3494,34 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>annual</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="n"/>
+          <t>annual DCF(5月1日测试,FY2022-2024未减值)</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>annual quantitative(2022/2023未减值)</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>annual(Q4定量测试,FY2023 SBU全额减值101)</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>annual Q4(FY2024未减值)</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>annual(2021-2023未减值)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
@@ -2691,7 +3572,31 @@
           <t>Intelligent Cloud/Productivity/More Personal Computing</t>
         </is>
       </c>
-      <c r="K45" s="4" t="n"/>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>CCG/DCAI/NEX/IFS(IDM代工)</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>DRAM/NAND存储</t>
+        </is>
+      </c>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>汽车/能源生成与存储/服务及其他</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
@@ -2742,7 +3647,31 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="K46" s="4" t="n"/>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N46" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O46" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2755,7 +3684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CG6"/>
+  <dimension ref="A1:CG11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4613,10 +5542,8 @@
       <c r="H6" s="4" t="n">
         <v>76421</v>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="I6" s="4" t="n">
+        <v>93780</v>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
@@ -4657,8 +5584,10 @@
       <c r="T6" s="4" t="n">
         <v>29510</v>
       </c>
-      <c r="U6" s="4" t="n">
-        <v>0</v>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="V6" s="4" t="n">
         <v>0</v>
@@ -4672,8 +5601,10 @@
       <c r="Y6" s="4" t="n">
         <v>44477</v>
       </c>
-      <c r="Z6" s="4" t="n">
-        <v>1286</v>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="AA6" s="4" t="n">
         <v>118548</v>
@@ -4688,15 +5619,11 @@
           <t>5-15</t>
         </is>
       </c>
-      <c r="AD6" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AE6" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="AD6" s="4" t="n">
+        <v>8163</v>
+      </c>
+      <c r="AE6" s="4" t="n">
+        <v>6532</v>
       </c>
       <c r="AF6" s="5" t="inlineStr">
         <is>
@@ -4775,7 +5702,7 @@
       </c>
       <c r="AU6" s="4" t="inlineStr">
         <is>
-          <t>annual</t>
+          <t>annual DCF(5月1日测试,FY2022-2024未减值)</t>
         </is>
       </c>
       <c r="AV6" s="4" t="inlineStr">
@@ -4823,10 +5750,8 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="BG6" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="BG6" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="BH6" s="4" t="n">
         <v>0.1121</v>
@@ -4890,26 +5815,1663 @@
         <v>0.5824</v>
       </c>
       <c r="CA6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="CB6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="CC6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="CD6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="CE6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CF6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CG6" s="4" t="inlineStr">
+        <is>
+          <t>高风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Oracle Corporation</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>2024-05-31</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>140976</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>21536</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>34818</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>13282</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>20989</v>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>5634</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>6890</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>62230</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>52961</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>10467</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>15353</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>1274</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <v>8915</v>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>3129</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>3010</v>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <v>6866</v>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA7" s="4" t="n">
+        <v>18673</v>
+      </c>
+      <c r="AB7" s="4" t="inlineStr">
+        <is>
+          <t>5(FY2023 Q1由4年延长,本期无变更)</t>
+        </is>
+      </c>
+      <c r="AC7" s="4" t="inlineStr">
+        <is>
+          <t>1-40</t>
+        </is>
+      </c>
+      <c r="AD7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AE7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AO7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS7" s="4" t="inlineStr">
+        <is>
+          <t>1-5(计算机/网络/机器设备)</t>
+        </is>
+      </c>
+      <c r="AT7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX7" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="CF6" s="4" t="n">
+      <c r="AY7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA7" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="BB7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BD7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF7" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BG7" s="4" t="n">
+        <v>404</v>
+      </c>
+      <c r="BH7" s="4" t="n">
+        <v>0.1453</v>
+      </c>
+      <c r="BI7" s="4" t="n">
+        <v>0.0222</v>
+      </c>
+      <c r="BJ7" s="4" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="BK7" s="4" t="n">
+        <v>0.4903</v>
+      </c>
+      <c r="BL7" s="4" t="n">
+        <v>0.4414</v>
+      </c>
+      <c r="BM7" s="4" t="n">
+        <v>0.1683</v>
+      </c>
+      <c r="BN7" s="4" t="n">
+        <v>0.1296</v>
+      </c>
+      <c r="BO7" s="4" t="n">
+        <v>0.3188</v>
+      </c>
+      <c r="BP7" s="4" t="n">
+        <v>0.3757</v>
+      </c>
+      <c r="BQ7" s="4" t="n">
+        <v>2.4592</v>
+      </c>
+      <c r="BR7" s="4" t="n">
+        <v>0.3815</v>
+      </c>
+      <c r="BS7" s="4" t="n">
+        <v>0.6185</v>
+      </c>
+      <c r="BT7" s="4" t="n">
+        <v>0.2989</v>
+      </c>
+      <c r="BU7" s="4" t="n">
+        <v>0.1528</v>
+      </c>
+      <c r="BV7" s="4" t="n">
+        <v>0.1976</v>
+      </c>
+      <c r="BW7" s="4" t="n">
+        <v>0.2616</v>
+      </c>
+      <c r="BX7" s="4" t="n">
+        <v>0.2387</v>
+      </c>
+      <c r="BY7" s="4" t="n">
+        <v>0.0602</v>
+      </c>
+      <c r="BZ7" s="4" t="n">
+        <v>-0.2104</v>
+      </c>
+      <c r="CA7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CB7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CC7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CF7" s="4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="CG7" s="4" t="inlineStr">
+        <is>
+          <t>中高风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Intel Corporation</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2023-12-30</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>191572</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>96647</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>194657</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>98010</v>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>51182</v>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>43442</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>4589</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>27591</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>54228</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>1675</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>93</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>-913</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>16046</v>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>7847</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>1755</v>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <v>25750</v>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="AA8" s="4" t="n">
+        <v>11471</v>
+      </c>
+      <c r="AB8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC8" s="4" t="inlineStr">
+        <is>
+          <t>10-25</t>
+        </is>
+      </c>
+      <c r="AD8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AE8" s="4" t="n">
+        <v>100033</v>
+      </c>
+      <c r="AF8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AO8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS8" s="4" t="inlineStr">
+        <is>
+          <t>3-8(2023-01部分生产设备由5延至8)</t>
+        </is>
+      </c>
+      <c r="AT8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU8" s="4" t="inlineStr">
+        <is>
+          <t>annual quantitative(2022/2023未减值)</t>
+        </is>
+      </c>
+      <c r="AV8" s="4" t="inlineStr">
+        <is>
+          <t>CCG/DCAI/NEX/IFS(IDM代工)</t>
+        </is>
+      </c>
+      <c r="AW8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AY8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="BA8" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="BB8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC8" s="4" t="n">
+        <v>4200</v>
+      </c>
+      <c r="BD8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE8" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF8" s="4" t="n">
+        <v>411</v>
+      </c>
+      <c r="BG8" s="4" t="n">
+        <v>-62</v>
+      </c>
+      <c r="BH8" s="4" t="n">
+        <v>0.08119999999999999</v>
+      </c>
+      <c r="BI8" s="4" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="BJ8" s="4" t="n">
+        <v>0.0092</v>
+      </c>
+      <c r="BK8" s="4" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="BL8" s="4" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="BM8" s="4" t="n">
+        <v>0.2959</v>
+      </c>
+      <c r="BN8" s="4" t="n">
+        <v>0.4748</v>
+      </c>
+      <c r="BO8" s="4" t="n">
+        <v>0.2664</v>
+      </c>
+      <c r="BP8" s="4" t="n">
+        <v>0.2831</v>
+      </c>
+      <c r="BQ8" s="4" t="n">
+        <v>0.5611</v>
+      </c>
+      <c r="BR8" s="4" t="n">
+        <v>0.5034999999999999</v>
+      </c>
+      <c r="BS8" s="4" t="n">
+        <v>0.4965</v>
+      </c>
+      <c r="BT8" s="4" t="n">
+        <v>4.6848</v>
+      </c>
+      <c r="BU8" s="4" t="n">
+        <v>0.5044999999999999</v>
+      </c>
+      <c r="BV8" s="4" t="n">
+        <v>0.0309</v>
+      </c>
+      <c r="BW8" s="4" t="n">
+        <v>0.4495</v>
+      </c>
+      <c r="BX8" s="4" t="n">
+        <v>-0.2948</v>
+      </c>
+      <c r="BY8" s="4" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="BZ8" s="4" t="n">
+        <v>0.0365</v>
+      </c>
+      <c r="CA8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CB8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="CC8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CD8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="CE8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="CF8" s="4" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="CG8" s="4" t="inlineStr">
+        <is>
+          <t>高风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Micron Technology, Inc.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2023-08-31</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>64254</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>37928</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>87585</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>49657</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>2464</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>404</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>1150</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>15540</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>-5833</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>-5745</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>177</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>3114</v>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V9" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>7670</v>
+      </c>
+      <c r="X9" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <v>7676</v>
+      </c>
+      <c r="Z9" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="AA9" s="4" t="n">
+        <v>1559</v>
+      </c>
+      <c r="AB9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC9" s="4" t="inlineStr">
+        <is>
+          <t>10-30</t>
+        </is>
+      </c>
+      <c r="AD9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AE9" s="4" t="n">
+        <v>65555</v>
+      </c>
+      <c r="AF9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM9" s="4" t="n">
+        <v>-1416</v>
+      </c>
+      <c r="AN9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AO9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS9" s="4" t="inlineStr">
+        <is>
+          <t>7(生产设备;其他≤7)</t>
+        </is>
+      </c>
+      <c r="AT9" s="4" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="AU9" s="4" t="inlineStr">
+        <is>
+          <t>annual(Q4定量测试,FY2023 SBU全额减值101)</t>
+        </is>
+      </c>
+      <c r="AV9" s="4" t="inlineStr">
+        <is>
+          <t>DRAM/NAND存储</t>
+        </is>
+      </c>
+      <c r="AW9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AY9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="BA9" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="BB9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BD9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE9" s="4" t="n">
+        <v>1831</v>
+      </c>
+      <c r="BF9" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BG9" s="4" t="n">
+        <v>171</v>
+      </c>
+      <c r="BH9" s="4" t="n">
+        <v>0.2022</v>
+      </c>
+      <c r="BI9" s="4" t="n">
+        <v>0.1194</v>
+      </c>
+      <c r="BJ9" s="4" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="BK9" s="4" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="BL9" s="4" t="n">
+        <v>0.0179</v>
+      </c>
+      <c r="BM9" s="4" t="n">
+        <v>0.2004</v>
+      </c>
+      <c r="BN9" s="4" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="BO9" s="4" t="n">
+        <v>0.2024</v>
+      </c>
+      <c r="BP9" s="4" t="n">
+        <v>0.2419</v>
+      </c>
+      <c r="BQ9" s="4" t="n">
+        <v>0.4097</v>
+      </c>
+      <c r="BR9" s="4" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="BS9" s="4" t="n">
+        <v>0.433</v>
+      </c>
+      <c r="BT9" s="4" t="n">
+        <v>-1.3149</v>
+      </c>
+      <c r="BU9" s="4" t="n">
+        <v>0.5903</v>
+      </c>
+      <c r="BV9" s="4" t="n">
+        <v>-0.3754</v>
+      </c>
+      <c r="BW9" s="4" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="BX9" s="4" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="BY9" s="4" t="n">
+        <v>-0.4948</v>
+      </c>
+      <c r="BZ9" s="4" t="n">
+        <v>-0.3639</v>
+      </c>
+      <c r="CA9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CB9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="CD9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="CE9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CF9" s="4" t="n">
         <v>4.2</v>
       </c>
-      <c r="CG6" s="4" t="inlineStr">
+      <c r="CG9" s="4" t="inlineStr">
         <is>
           <t>高风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Salesforce, Inc.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>2024-01-31</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>99823</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>3689</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>6841</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>3152</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>4209</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>490</v>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>5278</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>48620</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>34857</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>4136</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>5011</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>814</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>4906</v>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="n">
+        <v>1100</v>
+      </c>
+      <c r="X10" s="4" t="n">
+        <v>1869</v>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <v>736</v>
+      </c>
+      <c r="Z10" s="4" t="n">
+        <v>629</v>
+      </c>
+      <c r="AA10" s="4" t="n">
+        <v>10234</v>
+      </c>
+      <c r="AB10" s="4" t="inlineStr">
+        <is>
+          <t>3-5(计算机/设备/软件)</t>
+        </is>
+      </c>
+      <c r="AC10" s="4" t="inlineStr">
+        <is>
+          <t>10-40</t>
+        </is>
+      </c>
+      <c r="AD10" s="4" t="n">
+        <v>293</v>
+      </c>
+      <c r="AE10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AO10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS10" s="4" t="inlineStr">
+        <is>
+          <t>5(家具);租赁改良≤10</t>
+        </is>
+      </c>
+      <c r="AT10" s="4" t="inlineStr">
+        <is>
+          <t>3-5(随PPE软件类)</t>
+        </is>
+      </c>
+      <c r="AU10" s="4" t="inlineStr">
+        <is>
+          <t>annual Q4(FY2024未减值)</t>
+        </is>
+      </c>
+      <c r="AV10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ10" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="BA10" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="BB10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BD10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BG10" s="4" t="n">
+        <v>988</v>
+      </c>
+      <c r="BH10" s="4" t="n">
+        <v>0.2982</v>
+      </c>
+      <c r="BI10" s="4" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="BJ10" s="4" t="n">
+        <v>0.0187</v>
+      </c>
+      <c r="BK10" s="4" t="n">
+        <v>0.5399</v>
+      </c>
+      <c r="BL10" s="4" t="n">
+        <v>0.4871</v>
+      </c>
+      <c r="BM10" s="4" t="n">
+        <v>0.1407</v>
+      </c>
+      <c r="BN10" s="4" t="n">
+        <v>0.0211</v>
+      </c>
+      <c r="BO10" s="4" t="n">
+        <v>0.1995</v>
+      </c>
+      <c r="BP10" s="4" t="n">
+        <v>0.3492</v>
+      </c>
+      <c r="BQ10" s="4" t="n">
+        <v>9.4489</v>
+      </c>
+      <c r="BR10" s="4" t="n">
+        <v>0.4608</v>
+      </c>
+      <c r="BS10" s="4" t="n">
+        <v>0.5392</v>
+      </c>
+      <c r="BT10" s="4" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="BU10" s="4" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="BV10" s="4" t="n">
+        <v>0.1187</v>
+      </c>
+      <c r="BW10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BX10" s="4" t="n">
+        <v>0.2182</v>
+      </c>
+      <c r="BY10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF10" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="CG10" s="4" t="inlineStr">
+        <is>
+          <t>中风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>2023-12-31</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>106618</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>29725</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>41782</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>12057</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>3799</v>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>5791</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>178</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>253</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>96773</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <v>14974</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>8891</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>-5001</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>3969</v>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="4" t="n">
+        <v>3330</v>
+      </c>
+      <c r="X11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y11" s="4" t="n">
+        <v>8898</v>
+      </c>
+      <c r="Z11" s="4" t="n">
+        <v>464</v>
+      </c>
+      <c r="AA11" s="4" t="n">
+        <v>13256</v>
+      </c>
+      <c r="AB11" s="4" t="inlineStr">
+        <is>
+          <t>3-10(计算机设备与软件)</t>
+        </is>
+      </c>
+      <c r="AC11" s="4" t="inlineStr">
+        <is>
+          <t>15-30</t>
+        </is>
+      </c>
+      <c r="AD11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AE11" s="4" t="n">
+        <v>16372</v>
+      </c>
+      <c r="AF11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AO11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS11" s="4" t="inlineStr">
+        <is>
+          <t>3-15(机器/设备/车辆/家具;tooling 4-7)</t>
+        </is>
+      </c>
+      <c r="AT11" s="4" t="inlineStr">
+        <is>
+          <t>3-5(内部使用软件)</t>
+        </is>
+      </c>
+      <c r="AU11" s="4" t="inlineStr">
+        <is>
+          <t>annual(2021-2023未减值)</t>
+        </is>
+      </c>
+      <c r="AV11" s="4" t="inlineStr">
+        <is>
+          <t>汽车/能源生成与存储/服务及其他</t>
+        </is>
+      </c>
+      <c r="AW11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AZ11" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="BA11" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="BB11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BD11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BG11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH11" s="4" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="BI11" s="4" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="BJ11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK11" s="4" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="BL11" s="4" t="n">
+        <v>0.0024</v>
+      </c>
+      <c r="BM11" s="4" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="BN11" s="4" t="n">
+        <v>0.0919</v>
+      </c>
+      <c r="BO11" s="4" t="n">
+        <v>0.2993</v>
+      </c>
+      <c r="BP11" s="4" t="n">
+        <v>0.9077</v>
+      </c>
+      <c r="BQ11" s="4" t="n">
+        <v>3.2556</v>
+      </c>
+      <c r="BR11" s="4" t="n">
+        <v>0.2886</v>
+      </c>
+      <c r="BS11" s="4" t="n">
+        <v>0.7114</v>
+      </c>
+      <c r="BT11" s="4" t="n">
+        <v>0.3745</v>
+      </c>
+      <c r="BU11" s="4" t="n">
+        <v>0.2788</v>
+      </c>
+      <c r="BV11" s="4" t="n">
+        <v>0.1547</v>
+      </c>
+      <c r="BW11" s="4" t="n">
+        <v>0.1948</v>
+      </c>
+      <c r="BX11" s="4" t="n">
+        <v>0.376</v>
+      </c>
+      <c r="BY11" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ11" s="4" t="n">
+        <v>0.2427</v>
+      </c>
+      <c r="CA11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CB11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CF11" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="CG11" s="4" t="inlineStr">
+        <is>
+          <t>中高风险</t>
         </is>
       </c>
     </row>
@@ -4924,7 +7486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4935,6 +7497,11 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4978,6 +7545,31 @@
           <t>MSFT</t>
         </is>
       </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -5010,6 +7602,21 @@
       <c r="H2" s="4" t="n">
         <v>0.1121</v>
       </c>
+      <c r="I2" s="4" t="n">
+        <v>0.1453</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0.08119999999999999</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0.2022</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>0.2982</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0.112</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -5042,6 +7649,21 @@
       <c r="H3" s="4" t="n">
         <v>0.0297</v>
       </c>
+      <c r="I3" s="4" t="n">
+        <v>0.0222</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.1194</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0.0312</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -5076,6 +7698,23 @@
       <c r="H4" s="4" t="n">
         <v>0.0094</v>
       </c>
+      <c r="I4" s="4" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0.0092</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0.0187</v>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -5110,6 +7749,21 @@
       <c r="H5" s="4" t="n">
         <v>0.2867</v>
       </c>
+      <c r="I5" s="4" t="n">
+        <v>0.4903</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0.5399</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0.004</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -5142,6 +7796,21 @@
       <c r="H6" s="4" t="n">
         <v>0.2328</v>
       </c>
+      <c r="I6" s="4" t="n">
+        <v>0.4414</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0.0179</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0.4871</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -5174,6 +7843,21 @@
       <c r="H7" s="4" t="n">
         <v>0.1204</v>
       </c>
+      <c r="I7" s="4" t="n">
+        <v>0.1683</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0.2959</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0.2004</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>0.1407</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>0.041</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -5206,6 +7890,21 @@
       <c r="H8" s="4" t="n">
         <v>0.1814</v>
       </c>
+      <c r="I8" s="4" t="n">
+        <v>0.1296</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0.4748</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0.0211</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>0.0919</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -5238,6 +7937,21 @@
       <c r="H9" s="4" t="n">
         <v>0.328</v>
       </c>
+      <c r="I9" s="4" t="n">
+        <v>0.3188</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0.2664</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0.2024</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0.1995</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>0.2993</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -5270,6 +7984,21 @@
       <c r="H10" s="4" t="n">
         <v>0.4786</v>
       </c>
+      <c r="I10" s="4" t="n">
+        <v>0.3757</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0.2831</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0.2419</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0.3492</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0.9077</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -5302,6 +8031,21 @@
       <c r="H11" s="4" t="n">
         <v>1.8078</v>
       </c>
+      <c r="I11" s="4" t="n">
+        <v>2.4592</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0.5611</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0.4097</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>9.4489</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>3.2556</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -5334,6 +8078,21 @@
       <c r="H12" s="4" t="n">
         <v>0.3605</v>
       </c>
+      <c r="I12" s="4" t="n">
+        <v>0.3815</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0.5034999999999999</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0.4608</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0.2886</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -5366,6 +8125,21 @@
       <c r="H13" s="4" t="n">
         <v>0.6395</v>
       </c>
+      <c r="I13" s="4" t="n">
+        <v>0.6185</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0.4965</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>0.433</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>0.5392</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>0.7114</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -5380,7 +8154,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>depreciation/net_income</t>
+          <t>depreciation/net_income（TSLA特例：净利润含一次性递延税转回5.93B，改用operating_income口径）</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
@@ -5398,6 +8172,21 @@
       <c r="H14" s="4" t="n">
         <v>0.1725</v>
       </c>
+      <c r="I14" s="4" t="n">
+        <v>0.2989</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>4.6848</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>-1.3149</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0.3745</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -5430,6 +8219,21 @@
       <c r="H15" s="4" t="n">
         <v>0.2647</v>
       </c>
+      <c r="I15" s="4" t="n">
+        <v>0.1528</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0.5044999999999999</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>0.5903</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>0.2788</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -5462,6 +8266,21 @@
       <c r="H16" s="4" t="n">
         <v>0.3596</v>
       </c>
+      <c r="I16" s="4" t="n">
+        <v>0.1976</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0.0309</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>-0.3754</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0.1187</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>0.1547</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -5496,6 +8315,23 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="I17" s="4" t="n">
+        <v>0.2616</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0.4495</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="n">
+        <v>0.1948</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -5530,6 +8366,21 @@
       <c r="H18" s="4" t="n">
         <v>0.3818</v>
       </c>
+      <c r="I18" s="4" t="n">
+        <v>0.2387</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>-0.2948</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>0.2182</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>0.376</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -5570,6 +8421,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0602</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>-0.4948</v>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -5608,6 +8478,23 @@
       <c r="H20" s="4" t="n">
         <v>0.5824</v>
       </c>
+      <c r="I20" s="4" t="n">
+        <v>-0.2104</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0.0365</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>-0.3639</v>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0.2427</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5644,6 +8531,31 @@
         </is>
       </c>
       <c r="H21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -5660,7 +8572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6073,12 +8985,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>服务器/网络设备原值</t>
+          <t>服务器/网络设备净值</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>servers_gross</t>
+          <t>servers_net</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -6095,12 +9007,12 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>服务器/网络设备净值</t>
+          <t>建筑物净值</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>servers_net</t>
+          <t>buildings_net</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -6117,12 +9029,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>建筑物净值</t>
+          <t>在建工程</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>buildings_net</t>
+          <t>construction_in_progress</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -6139,17 +9051,633 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
+          <t>R&amp;D资本化金额</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>rd_capitalized</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>10-K正文</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>融资租赁本金支付</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>finance_lease_payments</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>合并现金流量表</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>服务器/网络设备净值</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>servers_net</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>建筑物原值</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>buildings_gross</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>建筑物净值</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>buildings_net</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>R&amp;D资本化金额</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>rd_capitalized</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>10-K正文</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>资产减值损失</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>impairment_loss</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>10-K正文</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>融资租赁本金支付</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>finance_lease_payments</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>合并现金流量表</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>服务器/网络设备原值</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>servers_gross</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>服务器/网络设备净值</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>servers_net</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>建筑物净值</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>buildings_net</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>R&amp;D资本化金额</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>rd_capitalized</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>10-K正文</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>服务器使用寿命</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>server_useful_life</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>附注1会计政策</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>服务器/网络设备原值</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>servers_gross</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>服务器/网络设备净值</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>servers_net</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>建筑物原值</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>buildings_gross</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>建筑物净值</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>buildings_net</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>R&amp;D资本化金额</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>rd_capitalized</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>10-K正文</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>服务器使用寿命</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>server_useful_life</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>附注1会计政策</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>服务器/网络设备净值</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>servers_net</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>建筑物净值</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>buildings_net</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
           <t>在建工程</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>construction_in_progress</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>R&amp;D资本化金额</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>rd_capitalized</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>10-K正文</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>资产减值损失</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>impairment_loss</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>10-K正文</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>服务器/网络设备净值</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>servers_net</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>建筑物原值</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>buildings_gross</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>建筑物净值</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>buildings_net</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>PP&amp;E附注(Note 7/10)表格</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>R&amp;D资本化金额</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>rd_capitalized</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>10-K正文</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>摊销费用</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>amortization</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>合并现金流量表</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MSFT scores updated to human-verified 5/4/3/4/5 -> 4.20; review_status confirmed for GOOGL/NVDA/AMD/MSFT; training set synced
</commit_message>
<xml_diff>
--- a/data/extracted/core_indicators_45_v01.xlsx
+++ b/data/extracted/core_indicators_45_v01.xlsx
@@ -5815,22 +5815,22 @@
         <v>0.5824</v>
       </c>
       <c r="CA6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="CB6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="CC6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="CD6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="CE6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="CF6" s="4" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="CG6" s="4" t="inlineStr">
         <is>

</xml_diff>